<commit_message>
Separar gráficos del análisis ABC para evitar solapamiento
Mueve el segundo gráfico (unidades vendidas) a la fila 36 para que
no se superponga con el primero (facturación), dejando espacio visual
entre ambos.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QBpwZC2zP5BKMd3Fa5CUTi
</commit_message>
<xml_diff>
--- a/Analisis_ABC_Productos.xlsx
+++ b/Analisis_ABC_Productos.xlsx
@@ -220,7 +220,6 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -372,7 +371,6 @@
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -640,7 +638,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>31</row>
+      <row>35</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="10080000" cy="5760000"/>

</xml_diff>

<commit_message>
Rehacer gráfico ABC como el modelo del profesor
Un único gráfico combinado con 4 series de barras (Unidades, Precio,
Facturación, % Facturación) más línea de % Acumulado en eje secundario,
productos en eje X ordenados por facturación descendente.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QBpwZC2zP5BKMd3Fa5CUTi
</commit_message>
<xml_diff>
--- a/Analisis_ABC_Productos.xlsx
+++ b/Analisis_ABC_Productos.xlsx
@@ -220,6 +220,7 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -230,7 +231,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Análisis ABC — Facturación y % Acumulado</a:t>
+              <a:t>Título del gráfico</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -245,12 +246,12 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Análisis ABC'!E3</f>
+              <f>'Análisis ABC'!C3</f>
             </strRef>
           </tx>
           <spPr>
             <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="1F4E79"/>
+              <a:srgbClr val="4472C4"/>
             </a:solidFill>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -258,12 +259,93 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Análisis ABC'!$B$4:$B$13</f>
+              <f>'Análisis ABC'!$A$4:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Análisis ABC'!$C$4:$C$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Análisis ABC'!D3</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="ED7D31"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Análisis ABC'!$A$4:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Análisis ABC'!$D$4:$D$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Análisis ABC'!E3</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="A5A5A5"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Análisis ABC'!$A$4:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
               <f>'Análisis ABC'!$E$4:$E$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'Análisis ABC'!F3</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="FFC000"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Análisis ABC'!$A$4:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Análisis ABC'!$F$4:$F$13</f>
             </numRef>
           </val>
         </ser>
@@ -274,17 +356,17 @@
       <lineChart>
         <grouping val="standard"/>
         <ser>
-          <idx val="1"/>
-          <order val="1"/>
+          <idx val="4"/>
+          <order val="4"/>
           <tx>
             <strRef>
               <f>'Análisis ABC'!G3</f>
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25000">
               <a:solidFill>
-                <a:srgbClr val="FF6600"/>
+                <a:srgbClr val="5B9BD5"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -312,21 +394,6 @@
           <orientation val="minMax"/>
         </scaling>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Productos</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -339,21 +406,6 @@
         </scaling>
         <axPos val="l"/>
         <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Facturación (€)</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -361,7 +413,7 @@
       </valAx>
     </plotArea>
     <legend>
-      <legendPos val="r"/>
+      <legendPos val="b"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -370,157 +422,6 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Análisis ABC — Unidades Vendidas y % Acumulado</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Análisis ABC'!C3</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="2E75B6"/>
-            </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Análisis ABC'!$B$4:$B$13</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Análisis ABC'!$C$4:$C$13</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <lineChart>
-        <grouping val="standard"/>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>'Análisis ABC'!G3</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28000">
-              <a:solidFill>
-                <a:srgbClr val="FF6600"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <val>
-            <numRef>
-              <f>'Análisis ABC'!$G$4:$G$13</f>
-            </numRef>
-          </val>
-        </ser>
-        <axId val="10"/>
-        <axId val="100"/>
-      </lineChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Productos</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Unidades vendidas</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-        <crosses val="min"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -619,7 +520,7 @@
       <row>15</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10080000" cy="5760000"/>
+    <ext cx="10800000" cy="6480000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -629,28 +530,6 @@
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>35</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="10080000" cy="5760000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="2" name="Chart 2"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>

</xml_diff>

<commit_message>
Añadir series ACUMULADO y PORCENTUAL al gráfico ABC
Gráfico con 6 series como el del profesor:
- 4 barras: Unidades vendidas (verde), Precio (rojo), TOTAL (verde claro),
  ACUMULADO (azul, suma acumulada en euros)
- 2 líneas: PORCENTUAL (morado, % individual) y % Acumulado (verde)
Eje izquierdo porcentajes 0-120%, eje derecho números 0-1.200.000.
Numeración 1-10 en eje X.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QBpwZC2zP5BKMd3Fa5CUTi
</commit_message>
<xml_diff>
--- a/Analisis_ABC_Productos.xlsx
+++ b/Analisis_ABC_Productos.xlsx
@@ -228,7 +228,7 @@
           </tx>
           <spPr>
             <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="4472C4"/>
+              <a:srgbClr val="00B050"/>
             </a:solidFill>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -255,7 +255,7 @@
           </tx>
           <spPr>
             <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="ED7D31"/>
+              <a:srgbClr val="FF0000"/>
             </a:solidFill>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -282,7 +282,7 @@
           </tx>
           <spPr>
             <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="A5A5A5"/>
+              <a:srgbClr val="92D050"/>
             </a:solidFill>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -309,7 +309,7 @@
           </tx>
           <spPr>
             <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="FFC000"/>
+              <a:srgbClr val="4472C4"/>
             </a:solidFill>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -343,7 +343,7 @@
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22000">
               <a:solidFill>
-                <a:srgbClr val="5B9BD5"/>
+                <a:srgbClr val="7030A0"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -359,6 +359,36 @@
           <val>
             <numRef>
               <f>'Hoja1'!$G$2:$G$11</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="5"/>
+          <order val="5"/>
+          <tx>
+            <strRef>
+              <f>'Hoja1'!H1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22000">
+              <a:solidFill>
+                <a:srgbClr val="00B050"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <val>
+            <numRef>
+              <f>'Hoja1'!$H$2:$H$11</f>
             </numRef>
           </val>
         </ser>
@@ -714,23 +744,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Código</t>
+          <t>Nº</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -750,30 +781,33 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Facturación</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>% Facturación</t>
+          <t>ACUMULADO</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>PORCENTUAL</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>% Acumulado</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Clasificación</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>P03</t>
-        </is>
+      <c r="A2" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
@@ -789,23 +823,24 @@
       <c r="E2" s="3" t="n">
         <v>150000</v>
       </c>
-      <c r="F2" s="4" t="n">
-        <v>0.15</v>
+      <c r="F2" s="3" t="n">
+        <v>150000</v>
       </c>
       <c r="G2" s="4" t="n">
         <v>0.15</v>
       </c>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="H2" s="4" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>P02</t>
-        </is>
+      <c r="A3" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
@@ -821,23 +856,24 @@
       <c r="E3" s="3" t="n">
         <v>250000</v>
       </c>
-      <c r="F3" s="4" t="n">
+      <c r="F3" s="3" t="n">
+        <v>400000</v>
+      </c>
+      <c r="G3" s="4" t="n">
         <v>0.25</v>
       </c>
-      <c r="G3" s="4" t="n">
+      <c r="H3" s="4" t="n">
         <v>0.4</v>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="I3" s="5" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>P01</t>
-        </is>
+      <c r="A4" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -853,23 +889,24 @@
       <c r="E4" s="3" t="n">
         <v>400000</v>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="F4" s="3" t="n">
+        <v>800000</v>
+      </c>
+      <c r="G4" s="4" t="n">
         <v>0.4</v>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="H4" s="4" t="n">
         <v>0.8</v>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>P04</t>
-        </is>
+      <c r="A5" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
@@ -885,23 +922,24 @@
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="F5" s="3" t="n">
+        <v>870000</v>
+      </c>
+      <c r="G5" s="4" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="G5" s="4" t="n">
+      <c r="H5" s="4" t="n">
         <v>0.87</v>
       </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="I5" s="6" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>P05</t>
-        </is>
+      <c r="A6" s="2" t="n">
+        <v>5</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
@@ -917,23 +955,24 @@
       <c r="E6" s="3" t="n">
         <v>50000</v>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="F6" s="3" t="n">
+        <v>920000</v>
+      </c>
+      <c r="G6" s="4" t="n">
         <v>0.05</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="H6" s="4" t="n">
         <v>0.92</v>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>P06</t>
-        </is>
+      <c r="A7" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
@@ -949,23 +988,24 @@
       <c r="E7" s="3" t="n">
         <v>30000</v>
       </c>
-      <c r="F7" s="4" t="n">
+      <c r="F7" s="3" t="n">
+        <v>950000</v>
+      </c>
+      <c r="G7" s="4" t="n">
         <v>0.03</v>
       </c>
-      <c r="G7" s="4" t="n">
+      <c r="H7" s="4" t="n">
         <v>0.95</v>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="I7" s="6" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>P07</t>
-        </is>
+      <c r="A8" s="2" t="n">
+        <v>7</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
@@ -981,23 +1021,24 @@
       <c r="E8" s="3" t="n">
         <v>20000</v>
       </c>
-      <c r="F8" s="4" t="n">
+      <c r="F8" s="3" t="n">
+        <v>970000</v>
+      </c>
+      <c r="G8" s="4" t="n">
         <v>0.02</v>
       </c>
-      <c r="G8" s="4" t="n">
+      <c r="H8" s="4" t="n">
         <v>0.97</v>
       </c>
-      <c r="H8" s="7" t="inlineStr">
+      <c r="I8" s="7" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>P08</t>
-        </is>
+      <c r="A9" s="2" t="n">
+        <v>8</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
@@ -1013,23 +1054,24 @@
       <c r="E9" s="3" t="n">
         <v>15000</v>
       </c>
-      <c r="F9" s="4" t="n">
+      <c r="F9" s="3" t="n">
+        <v>985000</v>
+      </c>
+      <c r="G9" s="4" t="n">
         <v>0.015</v>
       </c>
-      <c r="G9" s="4" t="n">
+      <c r="H9" s="4" t="n">
         <v>0.985</v>
       </c>
-      <c r="H9" s="7" t="inlineStr">
+      <c r="I9" s="7" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>P09</t>
-        </is>
+      <c r="A10" s="2" t="n">
+        <v>9</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
@@ -1045,23 +1087,24 @@
       <c r="E10" s="3" t="n">
         <v>10000</v>
       </c>
-      <c r="F10" s="4" t="n">
+      <c r="F10" s="3" t="n">
+        <v>995000</v>
+      </c>
+      <c r="G10" s="4" t="n">
         <v>0.01</v>
       </c>
-      <c r="G10" s="4" t="n">
+      <c r="H10" s="4" t="n">
         <v>0.995</v>
       </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="I10" s="7" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>P10</t>
-        </is>
+      <c r="A11" s="2" t="n">
+        <v>10</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
@@ -1077,13 +1120,16 @@
       <c r="E11" s="3" t="n">
         <v>5000</v>
       </c>
-      <c r="F11" s="4" t="n">
+      <c r="F11" s="3" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="G11" s="4" t="n">
         <v>0.005</v>
       </c>
-      <c r="G11" s="4" t="n">
+      <c r="H11" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="H11" s="7" t="inlineStr">
+      <c r="I11" s="7" t="inlineStr">
         <is>
           <t>C</t>
         </is>

</xml_diff>